<commit_message>
Prepare structure for Streamlit Cloud deployment
</commit_message>
<xml_diff>
--- a/log_book_final.xlsx
+++ b/log_book_final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/QXZ6BKI/work/logbook_deployment/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/QXZ6BKI/work/LOGBOOK_TEST/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152CD226-3DAC-D74E-A453-28AAAB5FFAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F43EEBAC-C721-5949-A2B1-9CCD84C2D2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -709,9 +709,6 @@
     <t>GZ_YIZHIAN_001</t>
   </si>
   <si>
-    <t>電裝壞筍</t>
-  </si>
-  <si>
     <t>周门充电站</t>
   </si>
   <si>
@@ -1616,8 +1613,11 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>測試結果</t>
+    <t>充电桩坏损</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Test Result</t>
   </si>
 </sst>
 </file>
@@ -1640,10 +1640,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color rgb="FFCE9178"/>
-      <name val="Microsoft JhengHei"/>
-      <family val="2"/>
+      <b/>
+      <sz val="11"/>
+      <name val="新細明體"/>
+      <family val="1"/>
       <charset val="136"/>
     </font>
   </fonts>
@@ -1655,12 +1655,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1669,7 +1684,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -2011,8 +2028,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="19" max="19" width="10" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="31.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="111.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="18">
+    <row r="1" spans="1:21">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2026,7 +2048,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -3762,7 +3784,7 @@
         <v>228</v>
       </c>
       <c r="U29" t="s">
-        <v>229</v>
+        <v>530</v>
       </c>
     </row>
     <row r="30" spans="1:21">
@@ -3773,7 +3795,7 @@
         <v>222</v>
       </c>
       <c r="C30" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D30" t="s">
         <v>41</v>
@@ -3782,22 +3804,22 @@
         <v>23</v>
       </c>
       <c r="F30" t="s">
+        <v>229</v>
+      </c>
+      <c r="G30" t="s">
         <v>230</v>
-      </c>
-      <c r="G30" t="s">
-        <v>231</v>
       </c>
       <c r="H30" t="s">
         <v>26</v>
       </c>
       <c r="I30" t="s">
+        <v>231</v>
+      </c>
+      <c r="J30" t="s">
         <v>232</v>
       </c>
-      <c r="J30" t="s">
+      <c r="K30" t="s">
         <v>233</v>
-      </c>
-      <c r="K30" t="s">
-        <v>234</v>
       </c>
       <c r="L30" t="s">
         <v>30</v>
@@ -3806,13 +3828,13 @@
         <v>31</v>
       </c>
       <c r="N30" t="s">
+        <v>234</v>
+      </c>
+      <c r="O30" t="s">
         <v>235</v>
       </c>
-      <c r="O30" t="s">
-        <v>236</v>
-      </c>
       <c r="P30" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="Q30" t="s">
         <v>197</v>
@@ -3824,7 +3846,7 @@
         <v>37</v>
       </c>
       <c r="U30" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" spans="1:21">
@@ -3835,7 +3857,7 @@
         <v>222</v>
       </c>
       <c r="C31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D31" t="s">
         <v>22</v>
@@ -3844,7 +3866,7 @@
         <v>23</v>
       </c>
       <c r="F31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G31" t="s">
         <v>49</v>
@@ -3868,13 +3890,13 @@
         <v>31</v>
       </c>
       <c r="N31" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="O31" t="s">
         <v>171</v>
       </c>
       <c r="P31" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Q31" t="s">
         <v>197</v>
@@ -3886,7 +3908,7 @@
         <v>37</v>
       </c>
       <c r="T31" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" spans="1:21">
@@ -3897,7 +3919,7 @@
         <v>222</v>
       </c>
       <c r="C32" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D32" t="s">
         <v>22</v>
@@ -3906,7 +3928,7 @@
         <v>23</v>
       </c>
       <c r="F32" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G32" t="s">
         <v>49</v>
@@ -3930,16 +3952,16 @@
         <v>31</v>
       </c>
       <c r="N32" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="O32" t="s">
         <v>197</v>
       </c>
       <c r="P32" t="s">
+        <v>242</v>
+      </c>
+      <c r="Q32" t="s">
         <v>243</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>244</v>
       </c>
       <c r="R32" t="s">
         <v>36</v>
@@ -3948,18 +3970,18 @@
         <v>37</v>
       </c>
       <c r="U32" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="33" spans="1:21">
       <c r="A33" t="s">
+        <v>245</v>
+      </c>
+      <c r="B33" t="s">
         <v>246</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>247</v>
-      </c>
-      <c r="C33" t="s">
-        <v>248</v>
       </c>
       <c r="D33" t="s">
         <v>31</v>
@@ -3971,7 +3993,7 @@
         <v>59</v>
       </c>
       <c r="G33" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H33" t="s">
         <v>61</v>
@@ -3986,22 +4008,22 @@
         <v>62</v>
       </c>
       <c r="L33" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="M33" t="s">
         <v>31</v>
       </c>
       <c r="N33" t="s">
+        <v>250</v>
+      </c>
+      <c r="O33" t="s">
         <v>251</v>
       </c>
-      <c r="O33" t="s">
+      <c r="P33" t="s">
         <v>252</v>
       </c>
-      <c r="P33" t="s">
-        <v>253</v>
-      </c>
       <c r="Q33" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="R33" t="s">
         <v>36</v>
@@ -4010,21 +4032,21 @@
         <v>37</v>
       </c>
       <c r="T33" t="s">
+        <v>253</v>
+      </c>
+      <c r="U33" t="s">
         <v>254</v>
-      </c>
-      <c r="U33" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="34" spans="1:21">
       <c r="A34" t="s">
+        <v>245</v>
+      </c>
+      <c r="B34" t="s">
         <v>246</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>247</v>
-      </c>
-      <c r="C34" t="s">
-        <v>248</v>
       </c>
       <c r="D34" t="s">
         <v>31</v>
@@ -4036,7 +4058,7 @@
         <v>59</v>
       </c>
       <c r="G34" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H34" t="s">
         <v>61</v>
@@ -4057,16 +4079,16 @@
         <v>31</v>
       </c>
       <c r="N34" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O34" t="s">
         <v>19</v>
       </c>
       <c r="P34" t="s">
+        <v>256</v>
+      </c>
+      <c r="Q34" t="s">
         <v>257</v>
-      </c>
-      <c r="Q34" t="s">
-        <v>258</v>
       </c>
       <c r="R34" t="s">
         <v>211</v>
@@ -4075,21 +4097,21 @@
         <v>37</v>
       </c>
       <c r="T34" t="s">
+        <v>253</v>
+      </c>
+      <c r="U34" t="s">
         <v>254</v>
-      </c>
-      <c r="U34" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="35" spans="1:21">
       <c r="A35" t="s">
+        <v>258</v>
+      </c>
+      <c r="B35" t="s">
         <v>259</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>260</v>
-      </c>
-      <c r="C35" t="s">
-        <v>261</v>
       </c>
       <c r="D35" t="s">
         <v>22</v>
@@ -4098,10 +4120,10 @@
         <v>23</v>
       </c>
       <c r="F35" t="s">
+        <v>261</v>
+      </c>
+      <c r="G35" t="s">
         <v>262</v>
-      </c>
-      <c r="G35" t="s">
-        <v>263</v>
       </c>
       <c r="H35" t="s">
         <v>61</v>
@@ -4122,16 +4144,16 @@
         <v>31</v>
       </c>
       <c r="N35" t="s">
+        <v>263</v>
+      </c>
+      <c r="O35" t="s">
         <v>264</v>
       </c>
-      <c r="O35" t="s">
+      <c r="P35" t="s">
         <v>265</v>
       </c>
-      <c r="P35" t="s">
-        <v>266</v>
-      </c>
       <c r="Q35" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="R35" t="s">
         <v>36</v>
@@ -4140,21 +4162,21 @@
         <v>37</v>
       </c>
       <c r="T35" t="s">
+        <v>266</v>
+      </c>
+      <c r="U35" t="s">
         <v>267</v>
-      </c>
-      <c r="U35" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="36" spans="1:21">
       <c r="A36" t="s">
+        <v>258</v>
+      </c>
+      <c r="B36" t="s">
         <v>259</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>260</v>
-      </c>
-      <c r="C36" t="s">
-        <v>261</v>
       </c>
       <c r="D36" t="s">
         <v>22</v>
@@ -4163,10 +4185,10 @@
         <v>23</v>
       </c>
       <c r="F36" t="s">
+        <v>261</v>
+      </c>
+      <c r="G36" t="s">
         <v>262</v>
-      </c>
-      <c r="G36" t="s">
-        <v>263</v>
       </c>
       <c r="H36" t="s">
         <v>61</v>
@@ -4187,16 +4209,16 @@
         <v>31</v>
       </c>
       <c r="N36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="O36" t="s">
         <v>100</v>
       </c>
       <c r="P36" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q36" t="s">
         <v>270</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>271</v>
       </c>
       <c r="R36" t="s">
         <v>36</v>
@@ -4205,21 +4227,21 @@
         <v>37</v>
       </c>
       <c r="T36" t="s">
+        <v>271</v>
+      </c>
+      <c r="U36" t="s">
         <v>272</v>
-      </c>
-      <c r="U36" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="37" spans="1:21">
       <c r="A37" t="s">
+        <v>258</v>
+      </c>
+      <c r="B37" t="s">
         <v>259</v>
       </c>
-      <c r="B37" t="s">
-        <v>260</v>
-      </c>
       <c r="C37" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D37" t="s">
         <v>73</v>
@@ -4228,10 +4250,10 @@
         <v>23</v>
       </c>
       <c r="F37" t="s">
+        <v>274</v>
+      </c>
+      <c r="G37" t="s">
         <v>275</v>
-      </c>
-      <c r="G37" t="s">
-        <v>276</v>
       </c>
       <c r="H37" t="s">
         <v>26</v>
@@ -4240,10 +4262,10 @@
         <v>27</v>
       </c>
       <c r="J37" t="s">
+        <v>276</v>
+      </c>
+      <c r="K37" t="s">
         <v>277</v>
-      </c>
-      <c r="K37" t="s">
-        <v>278</v>
       </c>
       <c r="L37" t="s">
         <v>30</v>
@@ -4252,16 +4274,16 @@
         <v>31</v>
       </c>
       <c r="N37" t="s">
+        <v>278</v>
+      </c>
+      <c r="O37" t="s">
+        <v>257</v>
+      </c>
+      <c r="P37" t="s">
         <v>279</v>
       </c>
-      <c r="O37" t="s">
-        <v>258</v>
-      </c>
-      <c r="P37" t="s">
+      <c r="Q37" t="s">
         <v>280</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>281</v>
       </c>
       <c r="R37" t="s">
         <v>36</v>
@@ -4270,21 +4292,21 @@
         <v>37</v>
       </c>
       <c r="T37" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="U37" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="38" spans="1:21">
       <c r="A38" t="s">
+        <v>258</v>
+      </c>
+      <c r="B38" t="s">
         <v>259</v>
       </c>
-      <c r="B38" t="s">
-        <v>260</v>
-      </c>
       <c r="C38" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D38" t="s">
         <v>96</v>
@@ -4293,10 +4315,10 @@
         <v>23</v>
       </c>
       <c r="F38" t="s">
+        <v>274</v>
+      </c>
+      <c r="G38" t="s">
         <v>275</v>
-      </c>
-      <c r="G38" t="s">
-        <v>276</v>
       </c>
       <c r="H38" t="s">
         <v>97</v>
@@ -4317,16 +4339,16 @@
         <v>31</v>
       </c>
       <c r="N38" t="s">
+        <v>282</v>
+      </c>
+      <c r="O38" t="s">
+        <v>280</v>
+      </c>
+      <c r="P38" t="s">
         <v>283</v>
       </c>
-      <c r="O38" t="s">
-        <v>281</v>
-      </c>
-      <c r="P38" t="s">
+      <c r="Q38" t="s">
         <v>284</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>285</v>
       </c>
       <c r="R38" t="s">
         <v>36</v>
@@ -4335,21 +4357,21 @@
         <v>37</v>
       </c>
       <c r="T38" t="s">
+        <v>285</v>
+      </c>
+      <c r="U38" t="s">
         <v>286</v>
-      </c>
-      <c r="U38" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="39" spans="1:21">
       <c r="A39" t="s">
+        <v>258</v>
+      </c>
+      <c r="B39" t="s">
         <v>259</v>
       </c>
-      <c r="B39" t="s">
-        <v>260</v>
-      </c>
       <c r="C39" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D39" t="s">
         <v>41</v>
@@ -4358,10 +4380,10 @@
         <v>23</v>
       </c>
       <c r="F39" t="s">
+        <v>288</v>
+      </c>
+      <c r="G39" t="s">
         <v>289</v>
-      </c>
-      <c r="G39" t="s">
-        <v>290</v>
       </c>
       <c r="H39" t="s">
         <v>26</v>
@@ -4370,7 +4392,7 @@
         <v>27</v>
       </c>
       <c r="J39" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="K39" t="s">
         <v>28</v>
@@ -4382,13 +4404,13 @@
         <v>31</v>
       </c>
       <c r="N39" t="s">
+        <v>291</v>
+      </c>
+      <c r="O39" t="s">
         <v>292</v>
       </c>
-      <c r="O39" t="s">
+      <c r="P39" t="s">
         <v>293</v>
-      </c>
-      <c r="P39" t="s">
-        <v>294</v>
       </c>
       <c r="Q39" t="s">
         <v>191</v>
@@ -4400,21 +4422,21 @@
         <v>37</v>
       </c>
       <c r="T39" t="s">
+        <v>294</v>
+      </c>
+      <c r="U39" t="s">
         <v>295</v>
-      </c>
-      <c r="U39" t="s">
-        <v>296</v>
       </c>
     </row>
     <row r="40" spans="1:21">
       <c r="A40" t="s">
+        <v>258</v>
+      </c>
+      <c r="B40" t="s">
         <v>259</v>
       </c>
-      <c r="B40" t="s">
-        <v>260</v>
-      </c>
       <c r="C40" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D40" t="s">
         <v>22</v>
@@ -4423,10 +4445,10 @@
         <v>23</v>
       </c>
       <c r="F40" t="s">
+        <v>297</v>
+      </c>
+      <c r="G40" t="s">
         <v>298</v>
-      </c>
-      <c r="G40" t="s">
-        <v>299</v>
       </c>
       <c r="H40" t="s">
         <v>26</v>
@@ -4435,10 +4457,10 @@
         <v>27</v>
       </c>
       <c r="J40" t="s">
+        <v>276</v>
+      </c>
+      <c r="K40" t="s">
         <v>277</v>
-      </c>
-      <c r="K40" t="s">
-        <v>278</v>
       </c>
       <c r="L40" t="s">
         <v>30</v>
@@ -4447,16 +4469,16 @@
         <v>31</v>
       </c>
       <c r="N40" t="s">
+        <v>299</v>
+      </c>
+      <c r="O40" t="s">
         <v>300</v>
       </c>
-      <c r="O40" t="s">
+      <c r="P40" t="s">
         <v>301</v>
       </c>
-      <c r="P40" t="s">
+      <c r="Q40" t="s">
         <v>302</v>
-      </c>
-      <c r="Q40" t="s">
-        <v>303</v>
       </c>
       <c r="R40" t="s">
         <v>36</v>
@@ -4465,18 +4487,18 @@
         <v>37</v>
       </c>
       <c r="T40" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="41" spans="1:21">
       <c r="A41" t="s">
+        <v>258</v>
+      </c>
+      <c r="B41" t="s">
         <v>259</v>
       </c>
-      <c r="B41" t="s">
-        <v>260</v>
-      </c>
       <c r="C41" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D41" t="s">
         <v>73</v>
@@ -4485,10 +4507,10 @@
         <v>23</v>
       </c>
       <c r="F41" t="s">
+        <v>305</v>
+      </c>
+      <c r="G41" t="s">
         <v>306</v>
-      </c>
-      <c r="G41" t="s">
-        <v>307</v>
       </c>
       <c r="H41" t="s">
         <v>26</v>
@@ -4509,16 +4531,16 @@
         <v>31</v>
       </c>
       <c r="N41" t="s">
+        <v>307</v>
+      </c>
+      <c r="O41" t="s">
         <v>308</v>
       </c>
-      <c r="O41" t="s">
+      <c r="P41" t="s">
         <v>309</v>
       </c>
-      <c r="P41" t="s">
+      <c r="Q41" t="s">
         <v>310</v>
-      </c>
-      <c r="Q41" t="s">
-        <v>311</v>
       </c>
       <c r="R41" t="s">
         <v>36</v>
@@ -4529,13 +4551,13 @@
     </row>
     <row r="42" spans="1:21">
       <c r="A42" t="s">
+        <v>258</v>
+      </c>
+      <c r="B42" t="s">
         <v>259</v>
       </c>
-      <c r="B42" t="s">
-        <v>260</v>
-      </c>
       <c r="C42" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D42" t="s">
         <v>41</v>
@@ -4544,10 +4566,10 @@
         <v>23</v>
       </c>
       <c r="F42" t="s">
+        <v>312</v>
+      </c>
+      <c r="G42" t="s">
         <v>313</v>
-      </c>
-      <c r="G42" t="s">
-        <v>314</v>
       </c>
       <c r="H42" t="s">
         <v>26</v>
@@ -4568,16 +4590,16 @@
         <v>31</v>
       </c>
       <c r="N42" t="s">
+        <v>314</v>
+      </c>
+      <c r="O42" t="s">
         <v>315</v>
       </c>
-      <c r="O42" t="s">
+      <c r="P42" t="s">
         <v>316</v>
       </c>
-      <c r="P42" t="s">
+      <c r="Q42" t="s">
         <v>317</v>
-      </c>
-      <c r="Q42" t="s">
-        <v>318</v>
       </c>
       <c r="R42" t="s">
         <v>140</v>
@@ -4586,18 +4608,18 @@
         <v>37</v>
       </c>
       <c r="T42" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="43" spans="1:21">
       <c r="A43" t="s">
+        <v>258</v>
+      </c>
+      <c r="B43" t="s">
         <v>259</v>
       </c>
-      <c r="B43" t="s">
-        <v>260</v>
-      </c>
       <c r="C43" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D43" t="s">
         <v>22</v>
@@ -4606,16 +4628,16 @@
         <v>23</v>
       </c>
       <c r="F43" t="s">
+        <v>319</v>
+      </c>
+      <c r="G43" t="s">
         <v>320</v>
-      </c>
-      <c r="G43" t="s">
-        <v>321</v>
       </c>
       <c r="H43" t="s">
         <v>26</v>
       </c>
       <c r="I43" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J43" t="s">
         <v>52</v>
@@ -4630,16 +4652,16 @@
         <v>31</v>
       </c>
       <c r="N43" t="s">
+        <v>322</v>
+      </c>
+      <c r="O43" t="s">
         <v>323</v>
       </c>
-      <c r="O43" t="s">
+      <c r="P43" t="s">
         <v>324</v>
       </c>
-      <c r="P43" t="s">
+      <c r="Q43" t="s">
         <v>325</v>
-      </c>
-      <c r="Q43" t="s">
-        <v>326</v>
       </c>
       <c r="R43" t="s">
         <v>36</v>
@@ -4648,18 +4670,18 @@
         <v>37</v>
       </c>
       <c r="T43" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="44" spans="1:21">
       <c r="A44" t="s">
+        <v>258</v>
+      </c>
+      <c r="B44" t="s">
         <v>259</v>
       </c>
-      <c r="B44" t="s">
-        <v>260</v>
-      </c>
       <c r="C44" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="D44" t="s">
         <v>22</v>
@@ -4668,16 +4690,16 @@
         <v>23</v>
       </c>
       <c r="F44" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G44" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H44" t="s">
         <v>26</v>
       </c>
       <c r="I44" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J44" t="s">
         <v>52</v>
@@ -4692,16 +4714,16 @@
         <v>31</v>
       </c>
       <c r="N44" t="s">
+        <v>328</v>
+      </c>
+      <c r="O44" t="s">
         <v>329</v>
       </c>
-      <c r="O44" t="s">
+      <c r="P44" t="s">
         <v>330</v>
       </c>
-      <c r="P44" t="s">
+      <c r="Q44" t="s">
         <v>331</v>
-      </c>
-      <c r="Q44" t="s">
-        <v>332</v>
       </c>
       <c r="R44" t="s">
         <v>36</v>
@@ -4710,18 +4732,18 @@
         <v>37</v>
       </c>
       <c r="T44" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="45" spans="1:21">
       <c r="A45" t="s">
+        <v>258</v>
+      </c>
+      <c r="B45" t="s">
         <v>259</v>
       </c>
-      <c r="B45" t="s">
-        <v>260</v>
-      </c>
       <c r="C45" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D45" t="s">
         <v>73</v>
@@ -4730,10 +4752,10 @@
         <v>23</v>
       </c>
       <c r="F45" t="s">
+        <v>334</v>
+      </c>
+      <c r="G45" t="s">
         <v>335</v>
-      </c>
-      <c r="G45" t="s">
-        <v>336</v>
       </c>
       <c r="H45" t="s">
         <v>26</v>
@@ -4751,16 +4773,16 @@
         <v>30</v>
       </c>
       <c r="M45" t="s">
+        <v>336</v>
+      </c>
+      <c r="N45" t="s">
         <v>337</v>
       </c>
-      <c r="N45" t="s">
+      <c r="O45" t="s">
+        <v>325</v>
+      </c>
+      <c r="P45" t="s">
         <v>338</v>
-      </c>
-      <c r="O45" t="s">
-        <v>326</v>
-      </c>
-      <c r="P45" t="s">
-        <v>339</v>
       </c>
       <c r="Q45" t="s">
         <v>35</v>
@@ -4772,18 +4794,18 @@
         <v>37</v>
       </c>
       <c r="T45" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="46" spans="1:21">
       <c r="A46" t="s">
+        <v>258</v>
+      </c>
+      <c r="B46" t="s">
         <v>259</v>
       </c>
-      <c r="B46" t="s">
-        <v>260</v>
-      </c>
       <c r="C46" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D46" t="s">
         <v>41</v>
@@ -4792,16 +4814,16 @@
         <v>23</v>
       </c>
       <c r="F46" t="s">
+        <v>305</v>
+      </c>
+      <c r="G46" t="s">
         <v>306</v>
-      </c>
-      <c r="G46" t="s">
-        <v>307</v>
       </c>
       <c r="H46" t="s">
         <v>26</v>
       </c>
       <c r="I46" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J46" t="s">
         <v>52</v>
@@ -4816,13 +4838,13 @@
         <v>31</v>
       </c>
       <c r="N46" t="s">
+        <v>341</v>
+      </c>
+      <c r="O46" t="s">
         <v>342</v>
       </c>
-      <c r="O46" t="s">
+      <c r="P46" t="s">
         <v>343</v>
-      </c>
-      <c r="P46" t="s">
-        <v>344</v>
       </c>
       <c r="Q46" t="s">
         <v>45</v>
@@ -4834,32 +4856,32 @@
         <v>37</v>
       </c>
       <c r="T46" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="47" spans="1:21">
       <c r="A47" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B47" t="s">
+        <v>345</v>
+      </c>
+      <c r="C47" t="s">
         <v>346</v>
       </c>
-      <c r="C47" t="s">
+      <c r="E47" t="s">
         <v>347</v>
-      </c>
-      <c r="E47" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="48" spans="1:21">
       <c r="A48" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B48" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C48" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D48" t="s">
         <v>41</v>
@@ -4868,10 +4890,10 @@
         <v>23</v>
       </c>
       <c r="F48" t="s">
+        <v>349</v>
+      </c>
+      <c r="G48" t="s">
         <v>350</v>
-      </c>
-      <c r="G48" t="s">
-        <v>351</v>
       </c>
       <c r="H48" t="s">
         <v>26</v>
@@ -4883,22 +4905,22 @@
         <v>52</v>
       </c>
       <c r="K48" t="s">
+        <v>351</v>
+      </c>
+      <c r="L48" t="s">
+        <v>30</v>
+      </c>
+      <c r="M48" t="s">
+        <v>336</v>
+      </c>
+      <c r="N48" t="s">
         <v>352</v>
       </c>
-      <c r="L48" t="s">
-        <v>30</v>
-      </c>
-      <c r="M48" t="s">
-        <v>337</v>
-      </c>
-      <c r="N48" t="s">
+      <c r="O48" t="s">
+        <v>342</v>
+      </c>
+      <c r="P48" t="s">
         <v>353</v>
-      </c>
-      <c r="O48" t="s">
-        <v>343</v>
-      </c>
-      <c r="P48" t="s">
-        <v>354</v>
       </c>
       <c r="Q48" t="s">
         <v>45</v>
@@ -4910,18 +4932,18 @@
         <v>37</v>
       </c>
       <c r="T48" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="49" spans="1:21">
       <c r="A49" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B49" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C49" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D49" t="s">
         <v>22</v>
@@ -4930,10 +4952,10 @@
         <v>23</v>
       </c>
       <c r="F49" t="s">
+        <v>356</v>
+      </c>
+      <c r="G49" t="s">
         <v>357</v>
-      </c>
-      <c r="G49" t="s">
-        <v>358</v>
       </c>
       <c r="H49" t="s">
         <v>26</v>
@@ -4951,19 +4973,19 @@
         <v>30</v>
       </c>
       <c r="M49" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N49" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="O49" t="s">
         <v>45</v>
       </c>
       <c r="P49" t="s">
+        <v>359</v>
+      </c>
+      <c r="Q49" t="s">
         <v>360</v>
-      </c>
-      <c r="Q49" t="s">
-        <v>361</v>
       </c>
       <c r="R49" t="s">
         <v>140</v>
@@ -4974,13 +4996,13 @@
     </row>
     <row r="50" spans="1:21">
       <c r="A50" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B50" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C50" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D50" t="s">
         <v>22</v>
@@ -4989,10 +5011,10 @@
         <v>23</v>
       </c>
       <c r="F50" t="s">
+        <v>362</v>
+      </c>
+      <c r="G50" t="s">
         <v>363</v>
-      </c>
-      <c r="G50" t="s">
-        <v>364</v>
       </c>
       <c r="H50" t="s">
         <v>26</v>
@@ -5001,7 +5023,7 @@
         <v>51</v>
       </c>
       <c r="J50" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="K50" t="s">
         <v>45</v>
@@ -5010,16 +5032,16 @@
         <v>30</v>
       </c>
       <c r="M50" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N50" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="O50" t="s">
         <v>45</v>
       </c>
       <c r="P50" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="Q50" t="s">
         <v>131</v>
@@ -5031,18 +5053,18 @@
         <v>37</v>
       </c>
       <c r="T50" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="51" spans="1:21">
       <c r="A51" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B51" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C51" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D51" t="s">
         <v>41</v>
@@ -5051,10 +5073,10 @@
         <v>23</v>
       </c>
       <c r="F51" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="G51" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H51" t="s">
         <v>26</v>
@@ -5072,16 +5094,16 @@
         <v>30</v>
       </c>
       <c r="M51" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N51" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="O51" t="s">
         <v>45</v>
       </c>
       <c r="P51" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="Q51" t="s">
         <v>45</v>
@@ -5093,18 +5115,18 @@
         <v>37</v>
       </c>
       <c r="T51" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="52" spans="1:21">
       <c r="A52" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B52" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C52" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D52" t="s">
         <v>96</v>
@@ -5113,10 +5135,10 @@
         <v>23</v>
       </c>
       <c r="F52" t="s">
+        <v>373</v>
+      </c>
+      <c r="G52" t="s">
         <v>374</v>
-      </c>
-      <c r="G52" t="s">
-        <v>375</v>
       </c>
       <c r="H52" t="s">
         <v>97</v>
@@ -5134,16 +5156,16 @@
         <v>30</v>
       </c>
       <c r="M52" t="s">
+        <v>375</v>
+      </c>
+      <c r="N52" t="s">
         <v>376</v>
-      </c>
-      <c r="N52" t="s">
-        <v>377</v>
       </c>
       <c r="O52" t="s">
         <v>33</v>
       </c>
       <c r="P52" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="Q52" t="s">
         <v>33</v>
@@ -5155,18 +5177,18 @@
         <v>37</v>
       </c>
       <c r="T52" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="53" spans="1:21">
       <c r="A53" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B53" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C53" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D53" t="s">
         <v>96</v>
@@ -5175,10 +5197,10 @@
         <v>23</v>
       </c>
       <c r="F53" t="s">
+        <v>312</v>
+      </c>
+      <c r="G53" t="s">
         <v>313</v>
-      </c>
-      <c r="G53" t="s">
-        <v>314</v>
       </c>
       <c r="H53" t="s">
         <v>26</v>
@@ -5196,16 +5218,16 @@
         <v>30</v>
       </c>
       <c r="M53" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N53" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="O53" t="s">
         <v>109</v>
       </c>
       <c r="P53" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="Q53" t="s">
         <v>109</v>
@@ -5219,10 +5241,10 @@
     </row>
     <row r="54" spans="1:21">
       <c r="B54" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C54" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="D54" t="s">
         <v>22</v>
@@ -5231,10 +5253,10 @@
         <v>23</v>
       </c>
       <c r="F54" t="s">
+        <v>380</v>
+      </c>
+      <c r="G54" t="s">
         <v>381</v>
-      </c>
-      <c r="G54" t="s">
-        <v>382</v>
       </c>
       <c r="H54" t="s">
         <v>26</v>
@@ -5243,7 +5265,7 @@
         <v>51</v>
       </c>
       <c r="J54" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="K54" t="s">
         <v>28</v>
@@ -5252,16 +5274,16 @@
         <v>30</v>
       </c>
       <c r="M54" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N54" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="O54" t="s">
         <v>109</v>
       </c>
       <c r="P54" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="Q54" t="s">
         <v>131</v>
@@ -5273,18 +5295,18 @@
         <v>37</v>
       </c>
       <c r="T54" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="55" spans="1:21">
       <c r="A55" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B55" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C55" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="D55" t="s">
         <v>22</v>
@@ -5293,19 +5315,19 @@
         <v>23</v>
       </c>
       <c r="F55" t="s">
+        <v>387</v>
+      </c>
+      <c r="G55" t="s">
         <v>388</v>
-      </c>
-      <c r="G55" t="s">
-        <v>389</v>
       </c>
       <c r="H55" t="s">
         <v>26</v>
       </c>
       <c r="I55" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J55" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="K55" t="s">
         <v>28</v>
@@ -5314,16 +5336,16 @@
         <v>30</v>
       </c>
       <c r="M55" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N55" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="O55" t="s">
         <v>35</v>
       </c>
       <c r="P55" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="Q55" t="s">
         <v>139</v>
@@ -5335,18 +5357,18 @@
         <v>37</v>
       </c>
       <c r="T55" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="56" spans="1:21">
       <c r="A56" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B56" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C56" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D56" t="s">
         <v>41</v>
@@ -5355,10 +5377,10 @@
         <v>23</v>
       </c>
       <c r="F56" t="s">
+        <v>373</v>
+      </c>
+      <c r="G56" t="s">
         <v>374</v>
-      </c>
-      <c r="G56" t="s">
-        <v>375</v>
       </c>
       <c r="H56" t="s">
         <v>26</v>
@@ -5376,16 +5398,16 @@
         <v>30</v>
       </c>
       <c r="M56" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N56" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="O56" t="s">
         <v>35</v>
       </c>
       <c r="P56" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="Q56" t="s">
         <v>139</v>
@@ -5397,10 +5419,10 @@
         <v>37</v>
       </c>
       <c r="T56" t="s">
+        <v>396</v>
+      </c>
+      <c r="U56" t="s">
         <v>397</v>
-      </c>
-      <c r="U56" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="57" spans="1:21">
@@ -5408,10 +5430,10 @@
         <v>100</v>
       </c>
       <c r="B57" t="s">
+        <v>398</v>
+      </c>
+      <c r="C57" t="s">
         <v>399</v>
-      </c>
-      <c r="C57" t="s">
-        <v>400</v>
       </c>
       <c r="D57" t="s">
         <v>41</v>
@@ -5420,10 +5442,10 @@
         <v>23</v>
       </c>
       <c r="F57" t="s">
+        <v>400</v>
+      </c>
+      <c r="G57" t="s">
         <v>401</v>
-      </c>
-      <c r="G57" t="s">
-        <v>402</v>
       </c>
       <c r="H57" t="s">
         <v>61</v>
@@ -5441,16 +5463,16 @@
         <v>30</v>
       </c>
       <c r="M57" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N57" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="O57" t="s">
         <v>109</v>
       </c>
       <c r="P57" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="Q57" t="s">
         <v>139</v>
@@ -5462,7 +5484,7 @@
         <v>37</v>
       </c>
       <c r="T57" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="58" spans="1:21">
@@ -5470,10 +5492,10 @@
         <v>100</v>
       </c>
       <c r="B58" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C58" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="D58" t="s">
         <v>22</v>
@@ -5482,40 +5504,40 @@
         <v>23</v>
       </c>
       <c r="F58" t="s">
+        <v>406</v>
+      </c>
+      <c r="G58" t="s">
         <v>407</v>
-      </c>
-      <c r="G58" t="s">
-        <v>408</v>
       </c>
       <c r="H58" t="s">
         <v>26</v>
       </c>
       <c r="I58" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J58" t="s">
         <v>28</v>
       </c>
       <c r="K58" t="s">
+        <v>408</v>
+      </c>
+      <c r="L58" t="s">
+        <v>30</v>
+      </c>
+      <c r="M58" t="s">
+        <v>336</v>
+      </c>
+      <c r="N58" t="s">
         <v>409</v>
       </c>
-      <c r="L58" t="s">
-        <v>30</v>
-      </c>
-      <c r="M58" t="s">
-        <v>337</v>
-      </c>
-      <c r="N58" t="s">
+      <c r="O58" t="s">
+        <v>360</v>
+      </c>
+      <c r="P58" t="s">
         <v>410</v>
       </c>
-      <c r="O58" t="s">
-        <v>361</v>
-      </c>
-      <c r="P58" t="s">
+      <c r="Q58" t="s">
         <v>411</v>
-      </c>
-      <c r="Q58" t="s">
-        <v>412</v>
       </c>
       <c r="R58" t="s">
         <v>36</v>
@@ -5524,7 +5546,7 @@
         <v>37</v>
       </c>
       <c r="T58" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="59" spans="1:21">
@@ -5532,10 +5554,10 @@
         <v>100</v>
       </c>
       <c r="B59" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C59" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D59" t="s">
         <v>73</v>
@@ -5544,10 +5566,10 @@
         <v>23</v>
       </c>
       <c r="F59" t="s">
+        <v>414</v>
+      </c>
+      <c r="G59" t="s">
         <v>415</v>
-      </c>
-      <c r="G59" t="s">
-        <v>416</v>
       </c>
       <c r="H59" t="s">
         <v>26</v>
@@ -5565,19 +5587,19 @@
         <v>30</v>
       </c>
       <c r="M59" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N59" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="O59" t="s">
         <v>55</v>
       </c>
       <c r="P59" t="s">
+        <v>417</v>
+      </c>
+      <c r="Q59" t="s">
         <v>418</v>
-      </c>
-      <c r="Q59" t="s">
-        <v>419</v>
       </c>
       <c r="R59" t="s">
         <v>81</v>
@@ -5586,7 +5608,7 @@
         <v>31</v>
       </c>
       <c r="T59" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="60" spans="1:21">
@@ -5594,19 +5616,19 @@
         <v>100</v>
       </c>
       <c r="B60" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C60" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D60" t="s">
         <v>96</v>
       </c>
       <c r="E60" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F60" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="61" spans="1:21">
@@ -5614,10 +5636,10 @@
         <v>100</v>
       </c>
       <c r="B61" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C61" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="D61" t="s">
         <v>41</v>
@@ -5626,10 +5648,10 @@
         <v>23</v>
       </c>
       <c r="F61" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="G61" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H61" t="s">
         <v>26</v>
@@ -5644,16 +5666,16 @@
         <v>30</v>
       </c>
       <c r="M61" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N61" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="O61" t="s">
         <v>45</v>
       </c>
       <c r="P61" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="Q61" t="s">
         <v>139</v>
@@ -5665,7 +5687,7 @@
         <v>31</v>
       </c>
       <c r="T61" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="62" spans="1:21">
@@ -5673,10 +5695,10 @@
         <v>100</v>
       </c>
       <c r="B62" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C62" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="D62" t="s">
         <v>22</v>
@@ -5685,10 +5707,10 @@
         <v>23</v>
       </c>
       <c r="F62" t="s">
+        <v>427</v>
+      </c>
+      <c r="G62" t="s">
         <v>428</v>
-      </c>
-      <c r="G62" t="s">
-        <v>429</v>
       </c>
       <c r="H62" t="s">
         <v>26</v>
@@ -5697,7 +5719,7 @@
         <v>27</v>
       </c>
       <c r="J62" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K62" t="s">
         <v>28</v>
@@ -5706,16 +5728,16 @@
         <v>30</v>
       </c>
       <c r="M62" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N62" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="O62" t="s">
         <v>91</v>
       </c>
       <c r="P62" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="Q62" t="s">
         <v>139</v>
@@ -5727,7 +5749,7 @@
         <v>37</v>
       </c>
       <c r="T62" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="63" spans="1:21">
@@ -5735,10 +5757,10 @@
         <v>100</v>
       </c>
       <c r="B63" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C63" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D63" t="s">
         <v>22</v>
@@ -5747,13 +5769,13 @@
         <v>23</v>
       </c>
       <c r="F63" t="s">
+        <v>433</v>
+      </c>
+      <c r="G63" t="s">
         <v>434</v>
       </c>
-      <c r="G63" t="s">
+      <c r="H63" t="s">
         <v>435</v>
-      </c>
-      <c r="H63" t="s">
-        <v>436</v>
       </c>
       <c r="I63" t="s">
         <v>51</v>
@@ -5768,16 +5790,16 @@
         <v>30</v>
       </c>
       <c r="M63" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N63" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="O63" t="s">
         <v>131</v>
       </c>
       <c r="P63" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="Q63" t="s">
         <v>139</v>
@@ -5789,7 +5811,7 @@
         <v>37</v>
       </c>
       <c r="T63" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="64" spans="1:21">
@@ -5797,10 +5819,10 @@
         <v>100</v>
       </c>
       <c r="B64" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C64" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D64" t="s">
         <v>22</v>
@@ -5809,10 +5831,10 @@
         <v>23</v>
       </c>
       <c r="F64" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="G64" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="H64" t="s">
         <v>26</v>
@@ -5830,16 +5852,16 @@
         <v>30</v>
       </c>
       <c r="M64" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N64" t="s">
+        <v>441</v>
+      </c>
+      <c r="O64" t="s">
+        <v>360</v>
+      </c>
+      <c r="P64" t="s">
         <v>442</v>
-      </c>
-      <c r="O64" t="s">
-        <v>361</v>
-      </c>
-      <c r="P64" t="s">
-        <v>443</v>
       </c>
       <c r="Q64" t="s">
         <v>139</v>
@@ -5851,7 +5873,7 @@
         <v>37</v>
       </c>
       <c r="T64" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="65" spans="1:21">
@@ -5859,33 +5881,33 @@
         <v>100</v>
       </c>
       <c r="B65" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C65" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D65" t="s">
         <v>96</v>
       </c>
       <c r="E65" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F65" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="U65" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="66" spans="1:21">
       <c r="A66" t="s">
+        <v>446</v>
+      </c>
+      <c r="B66" t="s">
         <v>447</v>
       </c>
-      <c r="B66" t="s">
-        <v>448</v>
-      </c>
       <c r="C66" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D66" t="s">
         <v>41</v>
@@ -5894,10 +5916,10 @@
         <v>23</v>
       </c>
       <c r="F66" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G66" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H66" t="s">
         <v>26</v>
@@ -5915,16 +5937,16 @@
         <v>30</v>
       </c>
       <c r="M66" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N66" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="O66" t="s">
         <v>45</v>
       </c>
       <c r="P66" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="Q66" t="s">
         <v>139</v>
@@ -5936,21 +5958,21 @@
         <v>37</v>
       </c>
       <c r="T66" t="s">
+        <v>451</v>
+      </c>
+      <c r="U66" t="s">
         <v>452</v>
-      </c>
-      <c r="U66" t="s">
-        <v>453</v>
       </c>
     </row>
     <row r="67" spans="1:21">
       <c r="A67" t="s">
+        <v>446</v>
+      </c>
+      <c r="B67" t="s">
         <v>447</v>
       </c>
-      <c r="B67" t="s">
-        <v>448</v>
-      </c>
       <c r="C67" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D67" t="s">
         <v>96</v>
@@ -5959,10 +5981,10 @@
         <v>23</v>
       </c>
       <c r="F67" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G67" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="H67" t="s">
         <v>26</v>
@@ -5971,19 +5993,19 @@
         <v>30</v>
       </c>
       <c r="M67" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N67" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="O67" t="s">
         <v>139</v>
       </c>
       <c r="P67" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="Q67" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="R67" t="s">
         <v>36</v>
@@ -5992,18 +6014,18 @@
         <v>37</v>
       </c>
       <c r="T67" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="68" spans="1:21">
       <c r="A68" t="s">
+        <v>446</v>
+      </c>
+      <c r="B68" t="s">
         <v>447</v>
       </c>
-      <c r="B68" t="s">
-        <v>448</v>
-      </c>
       <c r="C68" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D68" t="s">
         <v>22</v>
@@ -6012,10 +6034,10 @@
         <v>23</v>
       </c>
       <c r="F68" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="G68" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="H68" t="s">
         <v>61</v>
@@ -6033,19 +6055,19 @@
         <v>30</v>
       </c>
       <c r="M68" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N68" t="s">
+        <v>458</v>
+      </c>
+      <c r="O68" t="s">
+        <v>418</v>
+      </c>
+      <c r="P68" t="s">
         <v>459</v>
       </c>
-      <c r="O68" t="s">
-        <v>419</v>
-      </c>
-      <c r="P68" t="s">
+      <c r="Q68" t="s">
         <v>460</v>
-      </c>
-      <c r="Q68" t="s">
-        <v>461</v>
       </c>
       <c r="R68" t="s">
         <v>211</v>
@@ -6054,21 +6076,21 @@
         <v>37</v>
       </c>
       <c r="T68" t="s">
+        <v>461</v>
+      </c>
+      <c r="U68" t="s">
         <v>462</v>
-      </c>
-      <c r="U68" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="69" spans="1:21">
       <c r="A69" t="s">
+        <v>446</v>
+      </c>
+      <c r="B69" t="s">
         <v>447</v>
       </c>
-      <c r="B69" t="s">
-        <v>448</v>
-      </c>
       <c r="C69" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="D69" t="s">
         <v>96</v>
@@ -6077,10 +6099,10 @@
         <v>23</v>
       </c>
       <c r="F69" t="s">
+        <v>464</v>
+      </c>
+      <c r="G69" t="s">
         <v>465</v>
-      </c>
-      <c r="G69" t="s">
-        <v>466</v>
       </c>
       <c r="H69" t="s">
         <v>61</v>
@@ -6098,16 +6120,16 @@
         <v>30</v>
       </c>
       <c r="M69" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N69" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="O69" t="s">
         <v>65</v>
       </c>
       <c r="P69" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="Q69" t="s">
         <v>152</v>
@@ -6119,21 +6141,21 @@
         <v>37</v>
       </c>
       <c r="T69" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="U69" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="70" spans="1:21">
       <c r="A70" t="s">
+        <v>446</v>
+      </c>
+      <c r="B70" t="s">
         <v>447</v>
       </c>
-      <c r="B70" t="s">
-        <v>448</v>
-      </c>
       <c r="C70" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="D70" t="s">
         <v>22</v>
@@ -6142,10 +6164,10 @@
         <v>23</v>
       </c>
       <c r="F70" t="s">
+        <v>470</v>
+      </c>
+      <c r="G70" t="s">
         <v>471</v>
-      </c>
-      <c r="G70" t="s">
-        <v>472</v>
       </c>
       <c r="H70" t="s">
         <v>26</v>
@@ -6163,16 +6185,16 @@
         <v>30</v>
       </c>
       <c r="M70" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N70" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="O70" t="s">
         <v>146</v>
       </c>
       <c r="P70" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="Q70" t="s">
         <v>152</v>
@@ -6184,18 +6206,18 @@
         <v>37</v>
       </c>
       <c r="U70" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="71" spans="1:21">
       <c r="A71" t="s">
+        <v>446</v>
+      </c>
+      <c r="B71" t="s">
         <v>447</v>
       </c>
-      <c r="B71" t="s">
-        <v>448</v>
-      </c>
       <c r="C71" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D71" t="s">
         <v>96</v>
@@ -6204,10 +6226,10 @@
         <v>23</v>
       </c>
       <c r="F71" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="G71" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="H71" t="s">
         <v>26</v>
@@ -6219,25 +6241,25 @@
         <v>52</v>
       </c>
       <c r="K71" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="L71" t="s">
         <v>30</v>
       </c>
       <c r="M71" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N71" t="s">
+        <v>477</v>
+      </c>
+      <c r="O71" t="s">
+        <v>411</v>
+      </c>
+      <c r="P71" t="s">
         <v>478</v>
       </c>
-      <c r="O71" t="s">
-        <v>412</v>
-      </c>
-      <c r="P71" t="s">
+      <c r="Q71" t="s">
         <v>479</v>
-      </c>
-      <c r="Q71" t="s">
-        <v>480</v>
       </c>
       <c r="R71" t="s">
         <v>81</v>
@@ -6246,50 +6268,50 @@
         <v>37</v>
       </c>
       <c r="T71" t="s">
+        <v>480</v>
+      </c>
+      <c r="U71" t="s">
         <v>481</v>
-      </c>
-      <c r="U71" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="72" spans="1:21">
       <c r="A72" t="s">
+        <v>446</v>
+      </c>
+      <c r="B72" t="s">
         <v>447</v>
       </c>
-      <c r="B72" t="s">
-        <v>448</v>
-      </c>
       <c r="C72" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D72" t="s">
         <v>22</v>
       </c>
       <c r="E72" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="F72" t="s">
+        <v>335</v>
+      </c>
+      <c r="L72" t="s">
+        <v>30</v>
+      </c>
+      <c r="M72" t="s">
         <v>336</v>
       </c>
-      <c r="L72" t="s">
-        <v>30</v>
-      </c>
-      <c r="M72" t="s">
-        <v>337</v>
-      </c>
       <c r="U72" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="73" spans="1:21">
       <c r="A73" t="s">
+        <v>446</v>
+      </c>
+      <c r="B73" t="s">
         <v>447</v>
       </c>
-      <c r="B73" t="s">
-        <v>448</v>
-      </c>
       <c r="C73" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="D73" t="s">
         <v>22</v>
@@ -6298,37 +6320,37 @@
         <v>23</v>
       </c>
       <c r="F73" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="G73" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="H73" t="s">
         <v>26</v>
       </c>
       <c r="I73" t="s">
+        <v>484</v>
+      </c>
+      <c r="J73" t="s">
         <v>485</v>
       </c>
-      <c r="J73" t="s">
+      <c r="L73" t="s">
+        <v>30</v>
+      </c>
+      <c r="M73" t="s">
+        <v>336</v>
+      </c>
+      <c r="N73" t="s">
         <v>486</v>
       </c>
-      <c r="L73" t="s">
-        <v>30</v>
-      </c>
-      <c r="M73" t="s">
-        <v>337</v>
-      </c>
-      <c r="N73" t="s">
+      <c r="O73" t="s">
         <v>487</v>
       </c>
-      <c r="O73" t="s">
+      <c r="P73" t="s">
         <v>488</v>
       </c>
-      <c r="P73" t="s">
+      <c r="Q73" t="s">
         <v>489</v>
-      </c>
-      <c r="Q73" t="s">
-        <v>490</v>
       </c>
       <c r="R73" t="s">
         <v>140</v>
@@ -6337,21 +6359,21 @@
         <v>37</v>
       </c>
       <c r="T73" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="U73" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="74" spans="1:21">
       <c r="A74" t="s">
+        <v>446</v>
+      </c>
+      <c r="B74" t="s">
         <v>447</v>
       </c>
-      <c r="B74" t="s">
-        <v>448</v>
-      </c>
       <c r="C74" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D74" t="s">
         <v>96</v>
@@ -6360,10 +6382,10 @@
         <v>23</v>
       </c>
       <c r="F74" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G74" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="H74" t="s">
         <v>26</v>
@@ -6381,16 +6403,16 @@
         <v>30</v>
       </c>
       <c r="M74" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N74" t="s">
+        <v>492</v>
+      </c>
+      <c r="O74" t="s">
+        <v>489</v>
+      </c>
+      <c r="P74" t="s">
         <v>493</v>
-      </c>
-      <c r="O74" t="s">
-        <v>490</v>
-      </c>
-      <c r="P74" t="s">
-        <v>494</v>
       </c>
       <c r="Q74" t="s">
         <v>121</v>
@@ -6402,18 +6424,18 @@
         <v>37</v>
       </c>
       <c r="U74" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="75" spans="1:21">
       <c r="A75" t="s">
+        <v>446</v>
+      </c>
+      <c r="B75" t="s">
         <v>447</v>
       </c>
-      <c r="B75" t="s">
-        <v>448</v>
-      </c>
       <c r="C75" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D75" t="s">
         <v>96</v>
@@ -6422,10 +6444,10 @@
         <v>23</v>
       </c>
       <c r="F75" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G75" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="H75" t="s">
         <v>26</v>
@@ -6434,7 +6456,7 @@
         <v>30</v>
       </c>
       <c r="M75" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R75" t="s">
         <v>140</v>
@@ -6443,18 +6465,18 @@
         <v>193</v>
       </c>
       <c r="U75" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="76" spans="1:21">
       <c r="A76" t="s">
+        <v>446</v>
+      </c>
+      <c r="B76" t="s">
         <v>447</v>
       </c>
-      <c r="B76" t="s">
-        <v>448</v>
-      </c>
       <c r="C76" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="D76" t="s">
         <v>96</v>
@@ -6463,10 +6485,10 @@
         <v>23</v>
       </c>
       <c r="F76" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G76" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="H76" t="s">
         <v>26</v>
@@ -6484,19 +6506,19 @@
         <v>30</v>
       </c>
       <c r="M76" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N76" t="s">
+        <v>497</v>
+      </c>
+      <c r="O76" t="s">
+        <v>331</v>
+      </c>
+      <c r="P76" t="s">
         <v>498</v>
       </c>
-      <c r="O76" t="s">
-        <v>332</v>
-      </c>
-      <c r="P76" t="s">
-        <v>499</v>
-      </c>
       <c r="Q76" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="R76" t="s">
         <v>36</v>
@@ -6505,21 +6527,21 @@
         <v>37</v>
       </c>
       <c r="T76" t="s">
+        <v>499</v>
+      </c>
+      <c r="U76" t="s">
         <v>500</v>
-      </c>
-      <c r="U76" t="s">
-        <v>501</v>
       </c>
     </row>
     <row r="77" spans="1:21">
       <c r="A77" t="s">
+        <v>446</v>
+      </c>
+      <c r="B77" t="s">
         <v>447</v>
       </c>
-      <c r="B77" t="s">
-        <v>448</v>
-      </c>
       <c r="C77" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="D77" t="s">
         <v>96</v>
@@ -6528,10 +6550,10 @@
         <v>23</v>
       </c>
       <c r="F77" t="s">
+        <v>501</v>
+      </c>
+      <c r="G77" t="s">
         <v>502</v>
-      </c>
-      <c r="G77" t="s">
-        <v>503</v>
       </c>
       <c r="H77" t="s">
         <v>61</v>
@@ -6540,28 +6562,28 @@
         <v>51</v>
       </c>
       <c r="J77" t="s">
+        <v>503</v>
+      </c>
+      <c r="K77" t="s">
+        <v>503</v>
+      </c>
+      <c r="L77" t="s">
+        <v>30</v>
+      </c>
+      <c r="M77" t="s">
+        <v>336</v>
+      </c>
+      <c r="N77" t="s">
         <v>504</v>
       </c>
-      <c r="K77" t="s">
-        <v>504</v>
-      </c>
-      <c r="L77" t="s">
-        <v>30</v>
-      </c>
-      <c r="M77" t="s">
-        <v>337</v>
-      </c>
-      <c r="N77" t="s">
+      <c r="O77" t="s">
+        <v>489</v>
+      </c>
+      <c r="P77" t="s">
         <v>505</v>
       </c>
-      <c r="O77" t="s">
-        <v>490</v>
-      </c>
-      <c r="P77" t="s">
-        <v>506</v>
-      </c>
       <c r="Q77" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R77" t="s">
         <v>211</v>
@@ -6570,18 +6592,18 @@
         <v>37</v>
       </c>
       <c r="T77" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="78" spans="1:21">
       <c r="A78" t="s">
+        <v>446</v>
+      </c>
+      <c r="B78" t="s">
         <v>447</v>
       </c>
-      <c r="B78" t="s">
-        <v>448</v>
-      </c>
       <c r="C78" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="D78" t="s">
         <v>73</v>
@@ -6590,10 +6612,10 @@
         <v>23</v>
       </c>
       <c r="F78" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="G78" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="H78" t="s">
         <v>26</v>
@@ -6611,19 +6633,19 @@
         <v>30</v>
       </c>
       <c r="M78" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N78" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="O78" t="s">
         <v>99</v>
       </c>
       <c r="P78" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="Q78" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R78" t="s">
         <v>81</v>
@@ -6632,21 +6654,21 @@
         <v>37</v>
       </c>
       <c r="T78" t="s">
+        <v>510</v>
+      </c>
+      <c r="U78" t="s">
         <v>511</v>
-      </c>
-      <c r="U78" t="s">
-        <v>512</v>
       </c>
     </row>
     <row r="79" spans="1:21">
       <c r="A79" t="s">
+        <v>446</v>
+      </c>
+      <c r="B79" t="s">
         <v>447</v>
       </c>
-      <c r="B79" t="s">
-        <v>448</v>
-      </c>
       <c r="C79" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="D79" t="s">
         <v>22</v>
@@ -6655,10 +6677,10 @@
         <v>23</v>
       </c>
       <c r="F79" t="s">
+        <v>512</v>
+      </c>
+      <c r="G79" t="s">
         <v>513</v>
-      </c>
-      <c r="G79" t="s">
-        <v>514</v>
       </c>
       <c r="H79" t="s">
         <v>26</v>
@@ -6667,25 +6689,25 @@
         <v>51</v>
       </c>
       <c r="J79" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="K79" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="L79" t="s">
         <v>30</v>
       </c>
       <c r="M79" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N79" t="s">
+        <v>514</v>
+      </c>
+      <c r="O79" t="s">
+        <v>342</v>
+      </c>
+      <c r="P79" t="s">
         <v>515</v>
-      </c>
-      <c r="O79" t="s">
-        <v>343</v>
-      </c>
-      <c r="P79" t="s">
-        <v>516</v>
       </c>
       <c r="Q79" t="s">
         <v>33</v>
@@ -6697,21 +6719,21 @@
         <v>37</v>
       </c>
       <c r="T79" t="s">
+        <v>516</v>
+      </c>
+      <c r="U79" t="s">
         <v>517</v>
-      </c>
-      <c r="U79" t="s">
-        <v>518</v>
       </c>
     </row>
     <row r="80" spans="1:21">
       <c r="A80" t="s">
+        <v>446</v>
+      </c>
+      <c r="B80" t="s">
         <v>447</v>
       </c>
-      <c r="B80" t="s">
-        <v>448</v>
-      </c>
       <c r="C80" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D80" t="s">
         <v>22</v>
@@ -6720,10 +6742,10 @@
         <v>23</v>
       </c>
       <c r="F80" t="s">
+        <v>518</v>
+      </c>
+      <c r="G80" t="s">
         <v>519</v>
-      </c>
-      <c r="G80" t="s">
-        <v>520</v>
       </c>
       <c r="H80" t="s">
         <v>26</v>
@@ -6732,7 +6754,7 @@
         <v>27</v>
       </c>
       <c r="J80" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K80" t="s">
         <v>28</v>
@@ -6741,16 +6763,16 @@
         <v>30</v>
       </c>
       <c r="M80" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="N80" t="s">
+        <v>520</v>
+      </c>
+      <c r="O80" t="s">
+        <v>342</v>
+      </c>
+      <c r="P80" t="s">
         <v>521</v>
-      </c>
-      <c r="O80" t="s">
-        <v>343</v>
-      </c>
-      <c r="P80" t="s">
-        <v>522</v>
       </c>
       <c r="Q80" t="s">
         <v>35</v>
@@ -6762,21 +6784,21 @@
         <v>37</v>
       </c>
       <c r="T80" t="s">
+        <v>522</v>
+      </c>
+      <c r="U80" t="s">
         <v>523</v>
-      </c>
-      <c r="U80" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="81" spans="1:21">
       <c r="A81" t="s">
+        <v>446</v>
+      </c>
+      <c r="B81" t="s">
         <v>447</v>
       </c>
-      <c r="B81" t="s">
-        <v>448</v>
-      </c>
       <c r="C81" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="D81" t="s">
         <v>22</v>
@@ -6785,10 +6807,10 @@
         <v>23</v>
       </c>
       <c r="F81" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="G81" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H81" t="s">
         <v>26</v>
@@ -6806,16 +6828,16 @@
         <v>30</v>
       </c>
       <c r="M81" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="N81" t="s">
+        <v>525</v>
+      </c>
+      <c r="O81" t="s">
+        <v>342</v>
+      </c>
+      <c r="P81" t="s">
         <v>526</v>
-      </c>
-      <c r="O81" t="s">
-        <v>343</v>
-      </c>
-      <c r="P81" t="s">
-        <v>527</v>
       </c>
       <c r="Q81" t="s">
         <v>35</v>
@@ -6827,10 +6849,10 @@
         <v>37</v>
       </c>
       <c r="T81" t="s">
+        <v>527</v>
+      </c>
+      <c r="U81" t="s">
         <v>528</v>
-      </c>
-      <c r="U81" t="s">
-        <v>529</v>
       </c>
     </row>
   </sheetData>
@@ -6840,7 +6862,7 @@
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"BMWGroupTN Condensed"&amp;12&amp;KC00000 CONFIDENTIAL</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="A2:U81 A1:D1 F1:R1 T1:U1" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:U28 A1:D1 F1:R1 T1:U1 A30:U81 A29:T29" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>